<commit_message>
push perbaikan menu result setelah scan QR dan nambah menu untuk download rekap kehadiran tamu
</commit_message>
<xml_diff>
--- a/data/Daftar Tamu Undangan.xlsx
+++ b/data/Daftar Tamu Undangan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\app-qr-code-full-fixed\data\"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>No</t>
   </si>
@@ -31,12 +31,46 @@
   </si>
   <si>
     <t>Status Kehadiran</t>
+  </si>
+  <si>
+    <t>Ibu. Amaliyah &amp; Suami</t>
+  </si>
+  <si>
+    <t>25-Jul-2025 09:48:27</t>
+  </si>
+  <si>
+    <t>HADIR</t>
+  </si>
+  <si>
+    <t>Bpk. Eral &amp; Sipa</t>
+  </si>
+  <si>
+    <t>25-Jul-2025 09:53:29</t>
+  </si>
+  <si>
+    <t>Kel. Besar Bpk. KH. Hambali (Balaraja)</t>
+  </si>
+  <si>
+    <t>25-Jul-2025 10:02:45</t>
+  </si>
+  <si>
+    <t>Bpk. Syachroni &amp; Habibah</t>
+  </si>
+  <si>
+    <t>25-Jul-2025 10:11:57</t>
+  </si>
+  <si>
+    <t>Bpk. Ersa Yuda &amp; Nur Asiah</t>
+  </si>
+  <si>
+    <t>25-Jul-2025 10:13:19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="6">
     <font>
       <sz val="10"/>
@@ -533,13 +567,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="78.5703125" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="4.7109375"/>
+    <col min="2" max="2" customWidth="true" width="78.5703125"/>
+    <col min="3" max="3" customWidth="true" style="5" width="60.28515625"/>
+    <col min="4" max="4" customWidth="true" style="5" width="34.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75">
@@ -564,6 +598,61 @@
       <c r="B3" s="3"/>
       <c r="C3" s="6"/>
       <c r="D3" s="7"/>
+    </row>
+    <row r="4">
+      <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s" s="5">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s" s="5">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s" s="5">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s" s="5">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
clear data di excel
</commit_message>
<xml_diff>
--- a/data/Daftar Tamu Undangan.xlsx
+++ b/data/Daftar Tamu Undangan.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\app-qr-code-full-fixed\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\app-qr-code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>No</t>
   </si>
@@ -32,45 +32,11 @@
   <si>
     <t>Status Kehadiran</t>
   </si>
-  <si>
-    <t>Ibu. Amaliyah &amp; Suami</t>
-  </si>
-  <si>
-    <t>25-Jul-2025 09:48:27</t>
-  </si>
-  <si>
-    <t>HADIR</t>
-  </si>
-  <si>
-    <t>Bpk. Eral &amp; Sipa</t>
-  </si>
-  <si>
-    <t>25-Jul-2025 09:53:29</t>
-  </si>
-  <si>
-    <t>Kel. Besar Bpk. KH. Hambali (Balaraja)</t>
-  </si>
-  <si>
-    <t>25-Jul-2025 10:02:45</t>
-  </si>
-  <si>
-    <t>Bpk. Syachroni &amp; Habibah</t>
-  </si>
-  <si>
-    <t>25-Jul-2025 10:11:57</t>
-  </si>
-  <si>
-    <t>Bpk. Ersa Yuda &amp; Nur Asiah</t>
-  </si>
-  <si>
-    <t>25-Jul-2025 10:13:19</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="6">
     <font>
       <sz val="10"/>
@@ -570,10 +536,10 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="4.7109375"/>
-    <col min="2" max="2" customWidth="true" width="78.5703125"/>
-    <col min="3" max="3" customWidth="true" style="5" width="60.28515625"/>
-    <col min="4" max="4" customWidth="true" style="5" width="34.28515625"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="78.5703125" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75">
@@ -599,61 +565,11 @@
       <c r="C3" s="6"/>
       <c r="D3" s="7"/>
     </row>
-    <row r="4">
-      <c r="B4" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s" s="5">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s" s="5">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s" s="5">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s" s="5">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s" s="5">
-        <v>14</v>
-      </c>
-      <c r="D8" t="s" s="5">
-        <v>6</v>
-      </c>
-    </row>
+    <row r="4" spans="1:4" ht="12.75"/>
+    <row r="5" spans="1:4" ht="12.75"/>
+    <row r="6" spans="1:4" ht="12.75"/>
+    <row r="7" spans="1:4" ht="12.75"/>
+    <row r="8" spans="1:4" ht="12.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update JAR and target
</commit_message>
<xml_diff>
--- a/data/Daftar Tamu Undangan.xlsx
+++ b/data/Daftar Tamu Undangan.xlsx
@@ -533,13 +533,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="78.5703125" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="12.75">
@@ -565,11 +565,6 @@
       <c r="C3" s="6"/>
       <c r="D3" s="7"/>
     </row>
-    <row r="4" spans="1:4" ht="12.75"/>
-    <row r="5" spans="1:4" ht="12.75"/>
-    <row r="6" spans="1:4" ht="12.75"/>
-    <row r="7" spans="1:4" ht="12.75"/>
-    <row r="8" spans="1:4" ht="12.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>